<commit_message>
feat: update excess OT PDF generation with new column names and improved layout
</commit_message>
<xml_diff>
--- a/templates/excess_ot_template.xlsx
+++ b/templates/excess_ot_template.xlsx
@@ -27,24 +27,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00366092"/>
-        <bgColor rgb="00366092"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,17 +45,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,28 +425,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -465,144 +441,224 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>RH Hours</t>
+          <t>RH HOURS</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ND Hours</t>
+          <t>ND HOURS</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ROT Hours</t>
+          <t>ROT HOURS</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sunday/SPH Hours</t>
+          <t>SUNDAY HOURS</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Sunday/SPH OT Hours</t>
+          <t>SUN/SPH HOURS</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Sunday/SPH ND Hours</t>
+          <t>SUN/SPH OT HOURS</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>RH Pay</t>
+          <t>SUN/SPH ND HOURS</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ND Pay</t>
+          <t>RD+SPH HOURS</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>ROT Pay</t>
+          <t>RD+SPH OT HOURS</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Sunday/SPH Pay</t>
+          <t>RD+SPH ND HOURS</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Sunday/SPH OT Pay</t>
+          <t>OFFSET</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Sunday/SPH ND Pay</t>
+          <t>RH PAY</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>ND PAY</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>ROT PAY</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>SUNDAY PAY</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>SUN/SPH PAY</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>SUN/SPH OT PAY</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>SUN/SPH ND PAY</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>RD+SPH PAY</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>RD+SPH OT PAY</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>RD+SPH ND PAY</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>OFFSET Pay</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
           <t>Adjustment</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Total Pay</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Statement</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>December 16-31, 2025</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Doe, John</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dela Cruz, Juan</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="J2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="G2" s="2" t="n">
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="O2" t="n">
+        <v>300</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1500.5</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>800</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1560.52</v>
+      </c>
+      <c r="S2" t="n">
+        <v>250</v>
+      </c>
+      <c r="T2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="U2" t="n">
+        <v>600</v>
+      </c>
+      <c r="V2" t="n">
+        <v>350</v>
+      </c>
+      <c r="W2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="X2" t="n">
+        <v>150</v>
+      </c>
+      <c r="Y2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>1500.5</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>1560.52</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>3061.02</v>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>john.doe@example.com</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="Z2" t="n">
+        <v>6711.02</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>juan.delacruz@example.com</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>